<commit_message>
ajout calcul UFC quicksort
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_enzo.xlsx
+++ b/mesures/TP_mesures_enzo.xlsx
@@ -14,27 +14,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="139">
+  <si>
+    <t>Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
+  </si>
   <si>
     <t>Complexité cyclomatique (CC) - iqsort0</t>
   </si>
   <si>
-    <t>Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
-  </si>
-  <si>
-    <t>Nœuds</t>
-  </si>
-  <si>
-    <t>Arêtes</t>
+    <t>Métriques de Halstead - iqsort0</t>
   </si>
   <si>
     <t>Périmètre</t>
   </si>
   <si>
-    <t>Calcul de V(G) = E - N + 2P</t>
-  </si>
-  <si>
-    <t>Nœud</t>
+    <t>Opérateurs</t>
   </si>
   <si>
     <t>Fichiers</t>
@@ -43,10 +37,43 @@
     <t>LOC (lignes non vides)</t>
   </si>
   <si>
-    <t>Instruction</t>
+    <t>LOC moyen / fichier</t>
   </si>
   <si>
-    <t>LOC moyen / fichier</t>
+    <t>Opérandes</t>
+  </si>
+  <si>
+    <t>Dépôt complet (script scriptligne.sh)</t>
+  </si>
+  <si>
+    <t>Nœuds</t>
+  </si>
+  <si>
+    <t>Mesures</t>
+  </si>
+  <si>
+    <t>Arêtes</t>
+  </si>
+  <si>
+    <t>Opérateur</t>
+  </si>
+  <si>
+    <t>Calcul de V(G) = E - N + 2P</t>
+  </si>
+  <si>
+    <t>Occurrences</t>
+  </si>
+  <si>
+    <t>Opérande</t>
+  </si>
+  <si>
+    <t>Nœud</t>
+  </si>
+  <si>
+    <t>nt (opérateurs distincts)</t>
+  </si>
+  <si>
+    <t>Instruction</t>
   </si>
   <si>
     <t>Lignes</t>
@@ -55,16 +82,28 @@
     <t>De</t>
   </si>
   <si>
-    <t>Dépôt complet (script scriptligne.sh)</t>
-  </si>
-  <si>
     <t>Vers</t>
   </si>
   <si>
     <t>E (arêtes)</t>
   </si>
   <si>
+    <t>void</t>
+  </si>
+  <si>
+    <t>Score UFC</t>
+  </si>
+  <si>
     <t>Application ./app (php, js, jsx, css, ps1)</t>
+  </si>
+  <si>
+    <t>iqsort0</t>
+  </si>
+  <si>
+    <t>Nt (occurrences d'opérateurs)</t>
+  </si>
+  <si>
+    <t>Écart (Maquette, lockfile, etc.)</t>
   </si>
   <si>
     <t>N1</t>
@@ -76,10 +115,19 @@
     <t>3-4</t>
   </si>
   <si>
-    <t>Écart (Maquette, lockfile, etc.)</t>
+    <t>( )</t>
+  </si>
+  <si>
+    <t>swap</t>
   </si>
   <si>
     <t>N2</t>
+  </si>
+  <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
+    <t>nd (opérandes distincts)</t>
   </si>
   <si>
     <t>N (nœuds)</t>
@@ -94,31 +142,64 @@
     <t>Dépôt complet : exclut seulement .git, node_modules, .venv, __pycache__ (fichiers binaires ignorés).</t>
   </si>
   <si>
-    <t>return</t>
+    <t>int</t>
   </si>
   <si>
     <t>Application : find ./app sur *.php, *.js, *.jsx, *.css, *.ps1, hors node_modules et vendor.</t>
   </si>
   <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
+  </si>
+  <si>
+    <t>Calcul</t>
+  </si>
+  <si>
+    <t>Nd (occurrences d'opérandes)</t>
+  </si>
+  <si>
+    <t>Sous-total</t>
+  </si>
+  <si>
+    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
+  </si>
+  <si>
+    <t>return</t>
+  </si>
+  <si>
     <t>5</t>
+  </si>
+  <si>
+    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
   </si>
   <si>
     <t>N3</t>
   </si>
   <si>
+    <t>*</t>
+  </si>
+  <si>
     <t>P (composantes connexes)</t>
   </si>
   <si>
-    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
+    <t>n</t>
+  </si>
+  <si>
+    <t>Longueur N = Nt + Nd</t>
   </si>
   <si>
     <t>i = 1, j = 0</t>
   </si>
   <si>
+    <t>Poids (simple / moyen / difficile)</t>
+  </si>
+  <si>
     <t>6</t>
   </si>
   <si>
-    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
+    <t>Scores (simple / moyen / difficile)</t>
   </si>
   <si>
     <t>N9</t>
@@ -127,7 +208,43 @@
     <t>V(G) = E - N + 2P</t>
   </si>
   <si>
-    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
+    <t>Entrées externes</t>
+  </si>
+  <si>
+    <t>,</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>Vocabulaire n = nt + nd</t>
+  </si>
+  <si>
+    <t>3×4 + 4×3 + 6×1</t>
+  </si>
+  <si>
+    <t>1 / 2 / 4</t>
+  </si>
+  <si>
+    <t>1 / 1 / 0</t>
+  </si>
+  <si>
+    <t>1×1 + 2×1 + 4×0</t>
+  </si>
+  <si>
+    <t>{ }</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>Sorties externes</t>
+  </si>
+  <si>
+    <t>4×0 + 5×2 + 7×1</t>
+  </si>
+  <si>
+    <t>Volume = N * log2(n)</t>
   </si>
   <si>
     <t>N4</t>
@@ -136,7 +253,22 @@
     <t>i &lt; n ?</t>
   </si>
   <si>
+    <t>2 / 3 / 5</t>
+  </si>
+  <si>
+    <t>0 / 1 / 0</t>
+  </si>
+  <si>
+    <t>2×0 + 3×1 + 5×0</t>
+  </si>
+  <si>
     <t>Contrôle : décisions + 1 (3 décisions : lignes 4, 6, 7)</t>
+  </si>
+  <si>
+    <t>Requêtes externes</t>
+  </si>
+  <si>
+    <t>3×7 + 4×0 + 6×0</t>
   </si>
   <si>
     <t>N5</t>
@@ -145,7 +277,19 @@
     <t>a[i] &lt; a[0] ?</t>
   </si>
   <si>
+    <t>0 / 0 / 0</t>
+  </si>
+  <si>
     <t>7</t>
+  </si>
+  <si>
+    <t>1×0 + 2×0 + 4×0</t>
+  </si>
+  <si>
+    <t>Fichiers internes</t>
+  </si>
+  <si>
+    <t>7×3 + 10×0 + 15×0</t>
   </si>
   <si>
     <t>N6</t>
@@ -154,19 +298,59 @@
     <t>swap(++j, i, a)</t>
   </si>
   <si>
+    <t>3 / 5 / 8</t>
+  </si>
+  <si>
     <t>8</t>
+  </si>
+  <si>
+    <t>3×0 + 5×0 + 0×0</t>
+  </si>
+  <si>
+    <t>;</t>
   </si>
   <si>
     <t>N8</t>
   </si>
   <si>
+    <t>Fichiers externes</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>Contrôle : écart avec V(G)</t>
+  </si>
+  <si>
+    <t>5×0 + 7×5 + 10×2</t>
+  </si>
+  <si>
+    <t>Difficulté = (nt/2) * (Nd/nd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+3 / 5 / 8</t>
+  </si>
+  <si>
+    <t>3×0 + 5×0 + 8×0</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
   <si>
     <t>N7</t>
   </si>
   <si>
+    <t>if</t>
+  </si>
+  <si>
     <t>i++</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Effort = Difficulté * Volume</t>
   </si>
   <si>
     <t>swap + 2 appels iqsort0</t>
@@ -178,174 +362,27 @@
     <t>Hypothèses</t>
   </si>
   <si>
+    <t>Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
+Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
+Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
+  </si>
+  <si>
     <t>Sortie</t>
   </si>
   <si>
     <t>12</t>
   </si>
   <si>
-    <t>Métriques de Halstead - iqsort0</t>
+    <t>&lt;=</t>
   </si>
   <si>
     <t>P = 1 : une seule fonction, donc un seul graphe connexe.</t>
   </si>
   <si>
-    <t>Les 2 appels récursifs sont comptés dans le bloc N8 (pas de nœud de décision).</t>
+    <t>Conventions de comptage</t>
   </si>
   <si>
-    <t>Lignes : numérotation du code du sujet (void iqsort0 = ligne 1).</t>
-  </si>
-  <si>
-    <t>Valeurs en bleu : saisies ; valeurs en noir : formules.</t>
-  </si>
-  <si>
-    <t>Opérateurs</t>
-  </si>
-  <si>
-    <t>Opérandes</t>
-  </si>
-  <si>
-    <t>Mesures</t>
-  </si>
-  <si>
-    <t>Opérateur</t>
-  </si>
-  <si>
-    <t>Occurrences</t>
-  </si>
-  <si>
-    <t>Opérande</t>
-  </si>
-  <si>
-    <t>nt (opérateurs distincts)</t>
-  </si>
-  <si>
-    <t>void</t>
-  </si>
-  <si>
-    <t>iqsort0</t>
-  </si>
-  <si>
-    <t>Nt (occurrences d'opérateurs)</t>
-  </si>
-  <si>
-    <t>Score UFC</t>
-  </si>
-  <si>
-    <t>( )</t>
-  </si>
-  <si>
-    <t>swap</t>
-  </si>
-  <si>
-    <t>nd (opérandes distincts)</t>
-  </si>
-  <si>
-    <t>Catégorie</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>Nd (occurrences d'opérandes)</t>
-  </si>
-  <si>
-    <t>Calcul</t>
-  </si>
-  <si>
-    <t>Sous-total</t>
-  </si>
-  <si>
-    <t>Entrées externes</t>
-  </si>
-  <si>
-    <t>3×4 + 4×3 + 6×1</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>Sorties externes</t>
-  </si>
-  <si>
-    <t>4×0 + 5×2 + 7×1</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>Longueur N = Nt + Nd</t>
-  </si>
-  <si>
-    <t>Requêtes externes</t>
-  </si>
-  <si>
-    <t>3×7 + 4×0 + 6×0</t>
-  </si>
-  <si>
-    <t>Fichiers internes</t>
-  </si>
-  <si>
-    <t>7×3 + 10×0 + 15×0</t>
-  </si>
-  <si>
-    <t>Fichiers externes</t>
-  </si>
-  <si>
-    <t>5×0 + 7×5 + 10×2</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>,</t>
-  </si>
-  <si>
-    <t>i</t>
-  </si>
-  <si>
-    <t>Vocabulaire n = nt + nd</t>
-  </si>
-  <si>
-    <t>Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
-Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
-Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
-  </si>
-  <si>
-    <t>{ }</t>
-  </si>
-  <si>
-    <t>j</t>
-  </si>
-  <si>
-    <t>Volume = N * log2(n)</t>
-  </si>
-  <si>
-    <t>;</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>Difficulté = (nt/2) * (Nd/nd)</t>
-  </si>
-  <si>
-    <t>if</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Effort = Difficulté * Volume</t>
-  </si>
-  <si>
-    <t>&lt;=</t>
-  </si>
-  <si>
-    <t>Conventions de comptage</t>
+    <t>Les 2 appels récursifs sont comptés dans le bloc N8 (pas de nœud de décision).</t>
   </si>
   <si>
     <t>for</t>
@@ -354,10 +391,16 @@
     <t>Opérateurs : mots-clés (void, int, if, for, return), symboles (*, =, &lt;, &lt;=, +, -, ++), séparateurs (, ;).</t>
   </si>
   <si>
+    <t>Lignes : numérotation du code du sujet (void iqsort0 = ligne 1).</t>
+  </si>
+  <si>
     <t>=</t>
   </si>
   <si>
     <t>Les paires ( ), { } et [ ] comptent pour un seul opérateur chacune.</t>
+  </si>
+  <si>
+    <t>Valeurs en bleu : saisies ; valeurs en noir : formules.</t>
   </si>
   <si>
     <t>&lt;</t>
@@ -496,7 +539,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -506,10 +549,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -530,8 +573,14 @@
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -545,14 +594,11 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -801,7 +847,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -814,22 +860,22 @@
       <c r="D2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
+      <c r="A3" s="3" t="s">
+        <v>3</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="4" ht="15.0" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B4" s="6">
         <v>301.0</v>
@@ -844,7 +890,7 @@
     </row>
     <row r="5" ht="15.0" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="7">
@@ -854,7 +900,7 @@
     </row>
     <row r="6" ht="15.0" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="9">
@@ -870,8 +916,8 @@
       <c r="D7" s="2"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="3" t="s">
-        <v>23</v>
+      <c r="A8" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -879,7 +925,7 @@
     </row>
     <row r="9" ht="15.0" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -887,7 +933,7 @@
     </row>
     <row r="10" ht="15.0" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -895,7 +941,7 @@
     </row>
     <row r="11" ht="15.0" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -903,7 +949,7 @@
     </row>
     <row r="12" ht="15.0" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -911,7 +957,7 @@
     </row>
     <row r="13" ht="15.0" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -919,7 +965,7 @@
     </row>
     <row r="14" ht="15.0" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -6869,7 +6915,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6892,42 +6938,42 @@
       <c r="I2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>2</v>
+      <c r="A3" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="3" t="s">
-        <v>3</v>
+      <c r="E3" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="3" t="s">
-        <v>5</v>
+      <c r="H3" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I3" s="2"/>
     </row>
     <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>6</v>
+      <c r="A4" s="3" t="s">
+        <v>17</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>9</v>
+      <c r="B4" s="3" t="s">
+        <v>19</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
+      <c r="C4" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
+      <c r="E4" s="3" t="s">
+        <v>21</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>14</v>
+      <c r="F4" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="I4" s="5">
         <f>COUNTA(E5:E15)</f>
@@ -6936,24 +6982,24 @@
     </row>
     <row r="5" ht="15.0" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="6" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="5" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="I5" s="5">
         <f>COUNTA(A5:A13)</f>
@@ -6962,24 +7008,24 @@
     </row>
     <row r="6" ht="15.0" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="6" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="5" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="I6" s="6">
         <v>1.0</v>
@@ -6987,50 +7033,50 @@
     </row>
     <row r="7" ht="15.0" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="6" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="3" t="s">
-        <v>36</v>
+      <c r="H7" s="4" t="s">
+        <v>63</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="4">
         <f>I4-I5+2*I6</f>
         <v>4</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="6" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="5" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="I8" s="6">
         <v>4.0</v>
@@ -7038,20 +7084,20 @@
     </row>
     <row r="9" ht="15.0" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="6" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -7059,24 +7105,24 @@
     </row>
     <row r="10" ht="15.0" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>46</v>
+        <v>95</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="6" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="5" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="I10" s="5">
         <f>I7-I8</f>
@@ -7085,20 +7131,20 @@
     </row>
     <row r="11" ht="15.0" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>50</v>
+        <v>109</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="6" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -7106,47 +7152,47 @@
     </row>
     <row r="12" ht="15.0" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>51</v>
+        <v>112</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>52</v>
+        <v>113</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="6" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="3" t="s">
-        <v>53</v>
+      <c r="H12" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="I12" s="2"/>
     </row>
     <row r="13" ht="15.0" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>55</v>
+        <v>117</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="6" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="5" t="s">
-        <v>57</v>
+        <v>119</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -7156,14 +7202,14 @@
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="6" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="5" t="s">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -7173,14 +7219,14 @@
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="6" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="5" t="s">
-        <v>59</v>
+        <v>124</v>
       </c>
       <c r="I15" s="2"/>
     </row>
@@ -7193,7 +7239,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="5" t="s">
-        <v>60</v>
+        <v>127</v>
       </c>
       <c r="I16" s="2"/>
     </row>
@@ -18049,7 +18095,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -18070,38 +18116,38 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>61</v>
+      <c r="A3" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="3" t="s">
-        <v>62</v>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="3" t="s">
-        <v>63</v>
+      <c r="G3" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H3" s="2"/>
     </row>
     <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>64</v>
+      <c r="A4" s="3" t="s">
+        <v>13</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>65</v>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="4" t="s">
-        <v>66</v>
+      <c r="D4" s="3" t="s">
+        <v>16</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>65</v>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="5" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="H4" s="5">
         <f>COUNTA(A5:A21)</f>
@@ -18110,21 +18156,21 @@
     </row>
     <row r="5" ht="15.0" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="B5" s="6">
         <v>1.0</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="6" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="E5" s="6">
         <v>3.0</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="5" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="H5" s="5">
         <f>SUM(B5:B21)</f>
@@ -18133,21 +18179,21 @@
     </row>
     <row r="6" ht="15.0" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="B6" s="6">
         <v>8.0</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="6" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="E6" s="6">
         <v>2.0</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="5" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="H6" s="5">
         <f>COUNTA(D5:D12)</f>
@@ -18156,21 +18202,21 @@
     </row>
     <row r="7" ht="15.0" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="B7" s="6">
         <v>3.0</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="6" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="E7" s="6">
         <v>7.0</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="5" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="H7" s="5">
         <f>SUM(E5:E12)</f>
@@ -18179,21 +18225,21 @@
     </row>
     <row r="8" ht="15.0" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>83</v>
+        <v>54</v>
       </c>
       <c r="B8" s="6">
         <v>1.0</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="6" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="E8" s="6">
         <v>4.0</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="5" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="H8" s="5">
         <f>H5+H7</f>
@@ -18202,21 +18248,21 @@
     </row>
     <row r="9" ht="15.0" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="B9" s="6">
         <v>9.0</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="6" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="E9" s="6">
         <v>6.0</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="5" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="H9" s="5">
         <f>H4+H6</f>
@@ -18225,67 +18271,67 @@
     </row>
     <row r="10" ht="15.0" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="B10" s="6">
         <v>1.0</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="6" t="s">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="E10" s="6">
         <v>7.0</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="5" t="s">
-        <v>101</v>
+        <v>76</v>
       </c>
-      <c r="H10" s="17">
+      <c r="H10" s="13">
         <f>H8*LOG(H9,2)</f>
         <v>390.0839199</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B11" s="6">
         <v>8.0</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E11" s="6">
         <v>3.0</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
-      <c r="H11" s="17">
+      <c r="H11" s="13">
         <f>(H4/2)*(H7/H6)</f>
         <v>38.25</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B12" s="6">
         <v>2.0</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E12" s="6">
         <v>4.0</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H12" s="18">
         <f>H11*H10</f>
@@ -18294,7 +18340,7 @@
     </row>
     <row r="13" ht="15.0" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B13" s="6">
         <v>1.0</v>
@@ -18308,7 +18354,7 @@
     </row>
     <row r="14" ht="15.0" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="B14" s="6">
         <v>1.0</v>
@@ -18317,14 +18363,14 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="3" t="s">
-        <v>109</v>
+      <c r="G14" s="4" t="s">
+        <v>120</v>
       </c>
       <c r="H14" s="2"/>
     </row>
     <row r="15" ht="15.0" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="B15" s="6">
         <v>1.0</v>
@@ -18334,13 +18380,13 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="5" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="H15" s="2"/>
     </row>
     <row r="16" ht="15.0" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="B16" s="6">
         <v>2.0</v>
@@ -18350,13 +18396,13 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="5" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="H16" s="2"/>
     </row>
     <row r="17" ht="15.0" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B17" s="6">
         <v>2.0</v>
@@ -18366,13 +18412,13 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="5" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" ht="15.0" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B18" s="6">
         <v>2.0</v>
@@ -18382,13 +18428,13 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="5" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" ht="15.0" customHeight="1">
       <c r="A19" s="6" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B19" s="6">
         <v>2.0</v>
@@ -18398,13 +18444,13 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="5" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="6" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B20" s="6">
         <v>2.0</v>
@@ -18414,13 +18460,13 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="5" t="s">
-        <v>60</v>
+        <v>127</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="6" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B21" s="6">
         <v>2.0</v>
@@ -18433,28 +18479,28 @@
       <c r="H21" s="2"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="19" t="s">
-        <v>122</v>
+      <c r="A22" s="20" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="20"/>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="22"/>
+      <c r="A23" s="21"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="23"/>
     </row>
     <row r="24" ht="63.75" customHeight="1">
-      <c r="A24" s="16" t="s">
-        <v>123</v>
+      <c r="A24" s="19" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="25" ht="36.0" customHeight="1">
-      <c r="A25" s="16" t="s">
-        <v>124</v>
+      <c r="A25" s="19" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="26" ht="27.75" customHeight="1"/>
@@ -18464,14 +18510,14 @@
     <row r="30" ht="24.75" customHeight="1"/>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="16.5" customHeight="1">
-      <c r="A32" s="23"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
+      <c r="A32" s="24"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2"/>
@@ -28173,10 +28219,15 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="7" max="7" width="16.86"/>
+    <col customWidth="1" min="8" max="8" width="20.86"/>
+    <col customWidth="1" min="9" max="9" width="18.43"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -28184,108 +28235,226 @@
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="12">
+        <v>30.0</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="M4" s="12">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C5" s="12">
+        <v>17.0</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="I5" s="12" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="s">
+      <c r="K5" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="L5" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>82</v>
+      <c r="M5" s="12">
+        <v>3.0</v>
       </c>
-      <c r="C4" s="11">
-        <v>30.0</v>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="s">
+        <v>83</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>85</v>
+      <c r="C6" s="12">
+        <v>21.0</v>
       </c>
-      <c r="C5" s="11">
-        <v>17.0</v>
+      <c r="G6" s="12" t="s">
+        <v>83</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="s">
-        <v>88</v>
+      <c r="H6" s="12" t="s">
+        <v>69</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="I6" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="L6" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="11">
+      <c r="M6" s="12">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="12">
         <v>21.0</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="s">
+      <c r="G7" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>91</v>
+      <c r="H7" s="12" t="s">
+        <v>94</v>
       </c>
-      <c r="C7" s="11">
-        <v>21.0</v>
+      <c r="I7" s="12" t="s">
+        <v>87</v>
       </c>
+      <c r="K7" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="M7" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="s">
-        <v>92</v>
+      <c r="A8" s="12" t="s">
+        <v>99</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>93</v>
+      <c r="B8" s="12" t="s">
+        <v>102</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="12">
         <v>55.0</v>
       </c>
+      <c r="G8" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="M8" s="12">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="s">
-        <v>94</v>
+      <c r="A9" s="14" t="s">
+        <v>106</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="14">
+      <c r="B9" s="15"/>
+      <c r="C9" s="16">
         <v>144.0</v>
       </c>
+      <c r="G9" s="14"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="16"/>
+      <c r="K9" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L9" s="15"/>
+      <c r="M9" s="16">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="s">
-        <v>98</v>
+      <c r="A11" s="19" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
     </row>
     <row r="13">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
     </row>
     <row r="14">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
     </row>
     <row r="15">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Ajout COM et nouveau calcul MI
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_enzo.xlsx
+++ b/mesures/TP_mesures_enzo.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="151">
   <si>
     <t>Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
@@ -35,16 +35,13 @@
     <t>LOC moyen / fichier</t>
   </si>
   <si>
-    <t>Métriques de Halstead - iqsort0</t>
-  </si>
-  <si>
     <t>Dépôt complet (script scriptligne.sh)</t>
   </si>
   <si>
-    <t>Score UFC</t>
+    <t>Nœuds</t>
   </si>
   <si>
-    <t>Nœuds</t>
+    <t>Métriques de Halstead - iqsort0</t>
   </si>
   <si>
     <t>Arêtes</t>
@@ -56,7 +53,7 @@
     <t>Nœud</t>
   </si>
   <si>
-    <t>Catégorie</t>
+    <t>Score UFC</t>
   </si>
   <si>
     <t>Instruction</t>
@@ -83,12 +80,6 @@
     <t>Mesures</t>
   </si>
   <si>
-    <t>Calcul</t>
-  </si>
-  <si>
-    <t>Sous-total</t>
-  </si>
-  <si>
     <t>Opérateur</t>
   </si>
   <si>
@@ -98,7 +89,22 @@
     <t>Opérande</t>
   </si>
   <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
     <t>nt (opérateurs distincts)</t>
+  </si>
+  <si>
+    <t>Calcul</t>
+  </si>
+  <si>
+    <t>Sous-total</t>
+  </si>
+  <si>
+    <t>Application ./app (php, js, jsx, css, ps1)</t>
+  </si>
+  <si>
+    <t>Écart (Maquette, lockfile, etc.)</t>
   </si>
   <si>
     <t>Poids (simple / moyen / difficile)</t>
@@ -122,16 +128,28 @@
     <t>1×1 + 2×1 + 4×0</t>
   </si>
   <si>
-    <t>Application ./app (php, js, jsx, css, ps1)</t>
+    <t>Sorties externes</t>
   </si>
   <si>
-    <t>Sorties externes</t>
+    <t>N1</t>
+  </si>
+  <si>
+    <t>void</t>
   </si>
   <si>
     <t>4×0 + 5×2 + 7×1</t>
   </si>
   <si>
-    <t>Écart (Maquette, lockfile, etc.)</t>
+    <t>Méthode et hypothèses</t>
+  </si>
+  <si>
+    <t>if (n &lt;= 1)</t>
+  </si>
+  <si>
+    <t>3-4</t>
+  </si>
+  <si>
+    <t>iqsort0</t>
   </si>
   <si>
     <t>2 / 3 / 5</t>
@@ -140,28 +158,31 @@
     <t>0 / 1 / 0</t>
   </si>
   <si>
-    <t>N1</t>
+    <t>LOC = lignes non vides (commentaires inclus), mesurées avec le script bash scriptligne.sh.</t>
   </si>
   <si>
-    <t>if (n &lt;= 1)</t>
+    <t>Nt (occurrences d'opérateurs)</t>
+  </si>
+  <si>
+    <t>N2</t>
   </si>
   <si>
     <t>2×0 + 3×1 + 5×0</t>
   </si>
   <si>
-    <t>3-4</t>
+    <t>N (nœuds)</t>
+  </si>
+  <si>
+    <t>Dépôt complet : exclut seulement .git, node_modules, .venv, __pycache__ (fichiers binaires ignorés).</t>
   </si>
   <si>
     <t>Requêtes externes</t>
   </si>
   <si>
-    <t>N2</t>
-  </si>
-  <si>
     <t>3×7 + 4×0 + 6×0</t>
   </si>
   <si>
-    <t>N (nœuds)</t>
+    <t>Application : find ./app sur *.php, *.js, *.jsx, *.css, *.ps1, hors node_modules et vendor.</t>
   </si>
   <si>
     <t>0 / 0 / 0</t>
@@ -170,71 +191,68 @@
     <t>1×0 + 2×0 + 4×0</t>
   </si>
   <si>
-    <t>Méthode et hypothèses</t>
+    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
   </si>
   <si>
     <t>Fichiers internes</t>
   </si>
   <si>
-    <t>LOC = lignes non vides (commentaires inclus), mesurées avec le script bash scriptligne.sh.</t>
-  </si>
-  <si>
     <t>7×3 + 10×0 + 15×0</t>
   </si>
   <si>
-    <t>Dépôt complet : exclut seulement .git, node_modules, .venv, __pycache__ (fichiers binaires ignorés).</t>
+    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
   </si>
   <si>
     <t>3 / 5 / 8</t>
   </si>
   <si>
-    <t>Application : find ./app sur *.php, *.js, *.jsx, *.css, *.ps1, hors node_modules et vendor.</t>
-  </si>
-  <si>
     <t>3×0 + 5×0 + 0×0</t>
   </si>
   <si>
-    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
+    <t>return</t>
   </si>
   <si>
     <t>Fichiers externes</t>
   </si>
   <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>5×0 + 7×5 + 10×2</t>
   </si>
   <si>
-    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
-  </si>
-  <si>
-    <t>return</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
+    <t>N3</t>
   </si>
   <si>
     <t xml:space="preserve">
 3 / 5 / 8</t>
   </si>
   <si>
-    <t>N3</t>
+    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
+  </si>
+  <si>
+    <t>( )</t>
+  </si>
+  <si>
+    <t>P (composantes connexes)</t>
   </si>
   <si>
     <t>3×0 + 5×0 + 8×0</t>
   </si>
   <si>
-    <t>P (composantes connexes)</t>
-  </si>
-  <si>
-    <t>Total</t>
+    <t>swap</t>
   </si>
   <si>
     <t>i = 1, j = 0</t>
   </si>
   <si>
+    <t>nd (opérandes distincts)</t>
+  </si>
+  <si>
     <t>6</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
   <si>
     <t>N9</t>
@@ -243,24 +261,33 @@
     <t>V(G) = E - N + 2P</t>
   </si>
   <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>Nd (occurrences d'opérandes)</t>
+  </si>
+  <si>
     <t>Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
 Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
 Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
-  </si>
-  <si>
-    <t>void</t>
-  </si>
-  <si>
-    <t>iqsort0</t>
-  </si>
-  <si>
-    <t>Nt (occurrences d'opérateurs)</t>
   </si>
   <si>
     <t>N4</t>
   </si>
   <si>
     <t>i &lt; n ?</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>Longueur N = Nt + Nd</t>
   </si>
   <si>
     <t>Contrôle : décisions + 1 (3 décisions : lignes 4, 6, 7)</t>
@@ -281,31 +308,25 @@
     <t>swap(++j, i, a)</t>
   </si>
   <si>
-    <t>( )</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
-    <t>swap</t>
+    <t>,</t>
+  </si>
+  <si>
+    <t>i</t>
   </si>
   <si>
     <t>N8</t>
   </si>
   <si>
-    <t>nd (opérandes distincts)</t>
-  </si>
-  <si>
     <t>Contrôle : écart avec V(G)</t>
   </si>
   <si>
-    <t>int</t>
+    <t>Vocabulaire n = nt + nd</t>
   </si>
   <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>Nd (occurrences d'opérandes)</t>
+    <t>{ }</t>
   </si>
   <si>
     <t>N7</t>
@@ -314,13 +335,10 @@
     <t>i++</t>
   </si>
   <si>
-    <t>*</t>
+    <t>j</t>
   </si>
   <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>Longueur N = Nt + Nd</t>
+    <t>Volume = N * log2(n)</t>
   </si>
   <si>
     <t>swap + 2 appels iqsort0</t>
@@ -341,40 +359,22 @@
     <t>P = 1 : une seule fonction, donc un seul graphe connexe.</t>
   </si>
   <si>
-    <t>,</t>
-  </si>
-  <si>
-    <t>i</t>
-  </si>
-  <si>
-    <t>Vocabulaire n = nt + nd</t>
-  </si>
-  <si>
     <t>Les 2 appels récursifs sont comptés dans le bloc N8 (pas de nœud de décision).</t>
   </si>
   <si>
-    <t>{ }</t>
+    <t>;</t>
   </si>
   <si>
     <t>Lignes : numérotation du code du sujet (void iqsort0 = ligne 1).</t>
-  </si>
-  <si>
-    <t>j</t>
-  </si>
-  <si>
-    <t>Volume = N * log2(n)</t>
-  </si>
-  <si>
-    <t>Valeurs en bleu : saisies ; valeurs en noir : formules.</t>
-  </si>
-  <si>
-    <t>;</t>
   </si>
   <si>
     <t>0</t>
   </si>
   <si>
     <t>Difficulté = (nt/2) * (Nd/nd)</t>
+  </si>
+  <si>
+    <t>Valeurs en bleu : saisies ; valeurs en noir : formules.</t>
   </si>
   <si>
     <t>if</t>
@@ -456,6 +456,45 @@
   </si>
   <si>
     <t>171 - 5,2 * ln(390,08) - 0,23 * 4 - 16,2 * ln(12) + 0 = 171 − 31,03 − 0,92 − 40,26 ≈ 98,80</t>
+  </si>
+  <si>
+    <t>Calcul avec COM</t>
+  </si>
+  <si>
+    <t>0,52 ( 13 /24 )</t>
+  </si>
+  <si>
+    <t>171 - 5,2 * ln(390,08) - 0,23 * 4 - 16,2 * ln(12) + 50 * sin * sqrt(2,46 * 0,52 ) = 171 − 31,03 − 0,92 − 40,26 + 45,24  ≈ 144,04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On voit que le score est plus elevé avec les commentaires </t>
+  </si>
+  <si>
+    <t>/*
+ * Auteur      : Prénom NOM
+ * Date        : 08/10/2026
+ * Description : QuickSort simplifié (Bentley et McIlroy, 1993).
+ *               Trie en place les n premiers éléments du tableau a,
+ *               par ordre croissant.
+ */
+void iqsort0 ( int *a , int n )
+{
+    int i , j ;
+    // Cas de base : un tableau de 0 ou 1 élément est déjà trié
+    if ( n &lt;=1)
+        return ;
+    // Partitionnement autour du pivot a[0] : j = indice du dernier élément &lt; pivot
+    for ( i = 1 , j = 0; i &lt; n ; i ++)
+    // Si a[i] est plus petit que le pivot, on l'ajoute à la zone de gauche
+        if ( a [ i ] &lt; a [0])
+            swap (++ j , i , a );
+    // Place le pivot à sa position définitive j
+    swap (0 , j , a );
+    // Tri récursif de la partie gauche (éléments &lt; pivot)
+    iqsort0 (a , j );
+    // Tri récursif de la partie droite (éléments &gt;= pivot)
+    iqsort0 ( a + j +1 , n -j -1);
+}</t>
   </si>
 </sst>
 </file>
@@ -577,10 +616,10 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -589,14 +628,14 @@
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -907,22 +946,22 @@
     </row>
     <row r="4" ht="15.0" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>301.0</v>
       </c>
       <c r="C4" s="7">
         <v>23053.0</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="9">
         <f>C4/B4</f>
         <v>76.58803987</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="7">
@@ -932,7 +971,7 @@
     </row>
     <row r="6" ht="15.0" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="12">
@@ -948,8 +987,8 @@
       <c r="D7" s="2"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>51</v>
+      <c r="A8" s="5" t="s">
+        <v>41</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -957,7 +996,7 @@
     </row>
     <row r="9" ht="15.0" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -965,7 +1004,7 @@
     </row>
     <row r="10" ht="15.0" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -973,7 +1012,7 @@
     </row>
     <row r="11" ht="15.0" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -981,7 +1020,7 @@
     </row>
     <row r="12" ht="15.0" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -989,7 +1028,7 @@
     </row>
     <row r="13" ht="15.0" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -997,7 +1036,7 @@
     </row>
     <row r="14" ht="15.0" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -6970,42 +7009,42 @@
       <c r="I2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>9</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="6" t="s">
-        <v>10</v>
+      <c r="E3" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" ht="15.0" customHeight="1">
+      <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4">
         <f>COUNTA(E5:E15)</f>
@@ -7013,25 +7052,25 @@
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>41</v>
+      <c r="A5" s="6" t="s">
+        <v>38</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>44</v>
+      <c r="C5" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="5" t="s">
-        <v>41</v>
+      <c r="E5" s="6" t="s">
+        <v>38</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>46</v>
+      <c r="F5" s="6" t="s">
+        <v>49</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I5" s="4">
         <f>COUNTA(A5:A13)</f>
@@ -7039,122 +7078,122 @@
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>46</v>
+      <c r="A6" s="6" t="s">
+        <v>49</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>64</v>
       </c>
+      <c r="C6" s="6" t="s">
+        <v>66</v>
+      </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="5" t="s">
-        <v>41</v>
+      <c r="E6" s="6" t="s">
+        <v>38</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>67</v>
+      <c r="F6" s="6" t="s">
+        <v>68</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="5" t="s">
-        <v>67</v>
+      <c r="A7" s="6" t="s">
+        <v>68</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>71</v>
+      <c r="B7" s="6" t="s">
+        <v>75</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>72</v>
+      <c r="C7" s="6" t="s">
+        <v>77</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="5" t="s">
-        <v>46</v>
+      <c r="E7" s="6" t="s">
+        <v>49</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>73</v>
+      <c r="F7" s="6" t="s">
+        <v>79</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="6" t="s">
-        <v>74</v>
+      <c r="H7" s="5" t="s">
+        <v>80</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="5">
         <f>I4-I5+2*I6</f>
         <v>4</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="5" t="s">
-        <v>79</v>
+      <c r="A8" s="6" t="s">
+        <v>85</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>80</v>
+      <c r="B8" s="6" t="s">
+        <v>86</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>72</v>
+      <c r="C8" s="6" t="s">
+        <v>77</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="5" t="s">
-        <v>67</v>
+      <c r="E8" s="6" t="s">
+        <v>68</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>79</v>
+      <c r="F8" s="6" t="s">
+        <v>85</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="4" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="6">
         <v>4.0</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="5" t="s">
-        <v>82</v>
+      <c r="A9" s="6" t="s">
+        <v>91</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>83</v>
+      <c r="B9" s="6" t="s">
+        <v>92</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>84</v>
+      <c r="C9" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="5" t="s">
-        <v>79</v>
+      <c r="E9" s="6" t="s">
+        <v>85</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>82</v>
+      <c r="F9" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>90</v>
+      <c r="F10" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="4" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="I10" s="4">
         <f>I7-I8</f>
@@ -7162,69 +7201,69 @@
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="5" t="s">
-        <v>96</v>
+      <c r="A11" s="6" t="s">
+        <v>103</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>97</v>
+      <c r="B11" s="6" t="s">
+        <v>104</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>72</v>
+      <c r="C11" s="6" t="s">
+        <v>77</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="5" t="s">
-        <v>82</v>
+      <c r="E11" s="6" t="s">
+        <v>91</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>85</v>
+      <c r="F11" s="6" t="s">
+        <v>94</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="5" t="s">
-        <v>90</v>
+      <c r="A12" s="6" t="s">
+        <v>99</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>101</v>
+      <c r="B12" s="6" t="s">
+        <v>107</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>102</v>
+      <c r="C12" s="6" t="s">
+        <v>108</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="5" t="s">
-        <v>82</v>
+      <c r="E12" s="6" t="s">
+        <v>91</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>96</v>
+      <c r="F12" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="6" t="s">
-        <v>103</v>
+      <c r="H12" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="I12" s="2"/>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>73</v>
+      <c r="A13" s="6" t="s">
+        <v>79</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>104</v>
+      <c r="B13" s="6" t="s">
+        <v>110</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>105</v>
+      <c r="C13" s="6" t="s">
+        <v>111</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="5" t="s">
-        <v>85</v>
+      <c r="E13" s="6" t="s">
+        <v>94</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>96</v>
+      <c r="F13" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="4" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -7233,15 +7272,15 @@
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="5" t="s">
-        <v>96</v>
+      <c r="E14" s="6" t="s">
+        <v>103</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>79</v>
+      <c r="F14" s="6" t="s">
+        <v>85</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -7250,15 +7289,15 @@
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="5" t="s">
-        <v>90</v>
+      <c r="E15" s="6" t="s">
+        <v>99</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>73</v>
+      <c r="F15" s="6" t="s">
+        <v>79</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I15" s="2"/>
     </row>
@@ -7271,7 +7310,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I16" s="2"/>
     </row>
@@ -18127,7 +18166,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -18148,38 +18187,38 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>18</v>
+      <c r="A3" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="6" t="s">
-        <v>20</v>
+      <c r="D3" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" ht="15.0" customHeight="1">
+      <c r="A4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H4" s="4">
         <f>COUNTA(A5:A21)</f>
@@ -18187,22 +18226,22 @@
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>76</v>
+      <c r="A5" s="6" t="s">
+        <v>39</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="6">
         <v>1.0</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="5" t="s">
-        <v>77</v>
+      <c r="D5" s="6" t="s">
+        <v>44</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="6">
         <v>3.0</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="4" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="H5" s="4">
         <f>SUM(B5:B21)</f>
@@ -18210,22 +18249,22 @@
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>87</v>
+      <c r="A6" s="6" t="s">
+        <v>71</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="6">
         <v>8.0</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="5" t="s">
-        <v>89</v>
+      <c r="D6" s="6" t="s">
+        <v>74</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="6">
         <v>2.0</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="4" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="H6" s="4">
         <f>COUNTA(D5:D12)</f>
@@ -18233,22 +18272,22 @@
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="5" t="s">
-        <v>93</v>
+      <c r="A7" s="6" t="s">
+        <v>81</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="6">
         <v>3.0</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="5" t="s">
-        <v>94</v>
+      <c r="D7" s="6" t="s">
+        <v>82</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="6">
         <v>7.0</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="4" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="H7" s="4">
         <f>SUM(E5:E12)</f>
@@ -18256,22 +18295,22 @@
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="5" t="s">
-        <v>98</v>
+      <c r="A8" s="6" t="s">
+        <v>87</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="6">
         <v>1.0</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="5" t="s">
-        <v>99</v>
+      <c r="D8" s="6" t="s">
+        <v>88</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="6">
         <v>4.0</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="4" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="H8" s="4">
         <f>H5+H7</f>
@@ -18279,22 +18318,22 @@
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="5" t="s">
-        <v>107</v>
+      <c r="A9" s="6" t="s">
+        <v>97</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="6">
         <v>9.0</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="5" t="s">
-        <v>108</v>
+      <c r="D9" s="6" t="s">
+        <v>98</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="6">
         <v>6.0</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="4" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="H9" s="4">
         <f>H4+H6</f>
@@ -18302,22 +18341,22 @@
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="5" t="s">
-        <v>111</v>
+      <c r="A10" s="6" t="s">
+        <v>102</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="6">
         <v>1.0</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="5" t="s">
-        <v>113</v>
+      <c r="D10" s="6" t="s">
+        <v>105</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="6">
         <v>7.0</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="H10" s="18">
         <f>H8*LOG(H9,2)</f>
@@ -18325,22 +18364,22 @@
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="5" t="s">
-        <v>116</v>
+      <c r="A11" s="6" t="s">
+        <v>114</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="6">
         <v>8.0</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="5" t="s">
-        <v>117</v>
+      <c r="D11" s="6" t="s">
+        <v>116</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="6">
         <v>3.0</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H11" s="18">
         <f>(H4/2)*(H7/H6)</f>
@@ -18348,17 +18387,17 @@
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="6">
         <v>2.0</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="6">
         <v>4.0</v>
       </c>
       <c r="F12" s="2"/>
@@ -18371,10 +18410,10 @@
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="6">
         <v>1.0</v>
       </c>
       <c r="C13" s="2"/>
@@ -18385,26 +18424,26 @@
       <c r="H13" s="2"/>
     </row>
     <row r="14" ht="15.0" customHeight="1">
-      <c r="A14" s="5" t="s">
-        <v>63</v>
+      <c r="A14" s="6" t="s">
+        <v>64</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="6">
         <v>1.0</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="5" t="s">
         <v>123</v>
       </c>
       <c r="H14" s="2"/>
     </row>
     <row r="15" ht="15.0" customHeight="1">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="6">
         <v>1.0</v>
       </c>
       <c r="C15" s="2"/>
@@ -18417,10 +18456,10 @@
       <c r="H15" s="2"/>
     </row>
     <row r="16" ht="15.0" customHeight="1">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="6">
         <v>2.0</v>
       </c>
       <c r="C16" s="2"/>
@@ -18433,10 +18472,10 @@
       <c r="H16" s="2"/>
     </row>
     <row r="17" ht="15.0" customHeight="1">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="6">
         <v>2.0</v>
       </c>
       <c r="C17" s="2"/>
@@ -18449,10 +18488,10 @@
       <c r="H17" s="2"/>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="6">
         <v>2.0</v>
       </c>
       <c r="C18" s="2"/>
@@ -18465,10 +18504,10 @@
       <c r="H18" s="2"/>
     </row>
     <row r="19" ht="15.0" customHeight="1">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="6">
         <v>2.0</v>
       </c>
       <c r="C19" s="2"/>
@@ -18481,10 +18520,10 @@
       <c r="H19" s="2"/>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="6">
         <v>2.0</v>
       </c>
       <c r="C20" s="2"/>
@@ -18492,15 +18531,15 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="6">
         <v>2.0</v>
       </c>
       <c r="C21" s="2"/>
@@ -28259,7 +28298,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -28267,181 +28306,181 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>13</v>
+      <c r="G3" s="10" t="s">
+        <v>24</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>28</v>
+      <c r="H3" s="10" t="s">
+        <v>30</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>29</v>
+      <c r="I3" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
-        <v>30</v>
+      <c r="A4" s="11" t="s">
+        <v>32</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>31</v>
+      <c r="B4" s="11" t="s">
+        <v>33</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="11">
         <v>30.0</v>
       </c>
-      <c r="G4" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="10" t="s">
+      <c r="G4" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="L4" s="10" t="s">
+      <c r="H4" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="M4" s="10">
+      <c r="I4" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" s="11">
         <v>3.0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="10">
+      <c r="B5" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="11">
         <v>17.0</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>36</v>
+      <c r="G5" s="11" t="s">
+        <v>37</v>
       </c>
-      <c r="H5" s="10" t="s">
-        <v>39</v>
+      <c r="H5" s="11" t="s">
+        <v>45</v>
       </c>
-      <c r="I5" s="10" t="s">
-        <v>40</v>
+      <c r="I5" s="11" t="s">
+        <v>46</v>
       </c>
-      <c r="K5" s="10" t="s">
-        <v>36</v>
+      <c r="K5" s="11" t="s">
+        <v>37</v>
       </c>
-      <c r="L5" s="10" t="s">
-        <v>43</v>
+      <c r="L5" s="11" t="s">
+        <v>50</v>
       </c>
-      <c r="M5" s="10">
+      <c r="M5" s="11">
         <v>3.0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
-        <v>45</v>
+      <c r="A6" s="11" t="s">
+        <v>53</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>47</v>
+      <c r="B6" s="11" t="s">
+        <v>54</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="11">
         <v>21.0</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>45</v>
+      <c r="G6" s="11" t="s">
+        <v>53</v>
       </c>
-      <c r="H6" s="10" t="s">
-        <v>32</v>
+      <c r="H6" s="11" t="s">
+        <v>34</v>
       </c>
-      <c r="I6" s="10" t="s">
-        <v>49</v>
+      <c r="I6" s="11" t="s">
+        <v>56</v>
       </c>
-      <c r="K6" s="10" t="s">
-        <v>45</v>
+      <c r="K6" s="11" t="s">
+        <v>53</v>
       </c>
-      <c r="L6" s="10" t="s">
-        <v>50</v>
+      <c r="L6" s="11" t="s">
+        <v>57</v>
       </c>
-      <c r="M6" s="10">
+      <c r="M6" s="11">
         <v>0.0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="s">
-        <v>52</v>
+      <c r="A7" s="11" t="s">
+        <v>59</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>54</v>
+      <c r="B7" s="11" t="s">
+        <v>60</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="11">
         <v>21.0</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>52</v>
+      <c r="G7" s="11" t="s">
+        <v>59</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="10" t="s">
-        <v>49</v>
+      <c r="K7" s="11" t="s">
+        <v>59</v>
       </c>
-      <c r="K7" s="10" t="s">
-        <v>52</v>
+      <c r="L7" s="11" t="s">
+        <v>63</v>
       </c>
-      <c r="L7" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="M7" s="10">
+      <c r="M7" s="11">
         <v>0.0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="s">
-        <v>60</v>
+      <c r="A8" s="11" t="s">
+        <v>65</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>61</v>
+      <c r="B8" s="11" t="s">
+        <v>67</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="11">
         <v>55.0</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>60</v>
+      <c r="G8" s="11" t="s">
+        <v>65</v>
       </c>
-      <c r="H8" s="10" t="s">
-        <v>66</v>
+      <c r="H8" s="11" t="s">
+        <v>69</v>
       </c>
-      <c r="I8" s="10" t="s">
-        <v>49</v>
+      <c r="I8" s="11" t="s">
+        <v>56</v>
       </c>
-      <c r="K8" s="10" t="s">
-        <v>60</v>
+      <c r="K8" s="11" t="s">
+        <v>65</v>
       </c>
-      <c r="L8" s="10" t="s">
-        <v>68</v>
+      <c r="L8" s="11" t="s">
+        <v>73</v>
       </c>
-      <c r="M8" s="10">
+      <c r="M8" s="11">
         <v>0.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="15">
@@ -28451,7 +28490,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="15"/>
       <c r="K9" s="13" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="L9" s="14"/>
       <c r="M9" s="15">
@@ -28465,7 +28504,7 @@
     </row>
     <row r="11">
       <c r="A11" s="17" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12">
@@ -28510,7 +28549,7 @@
     </row>
     <row r="7">
       <c r="A7" s="25" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
@@ -28527,33 +28566,109 @@
       <c r="F9" s="26" t="s">
         <v>141</v>
       </c>
+      <c r="J9" s="26">
+        <v>390.08</v>
+      </c>
     </row>
     <row r="10">
       <c r="F10" s="26" t="s">
         <v>142</v>
       </c>
+      <c r="J10" s="26">
+        <v>4.0</v>
+      </c>
     </row>
     <row r="11">
       <c r="F11" s="26" t="s">
         <v>143</v>
       </c>
+      <c r="J11" s="26">
+        <v>12.0</v>
+      </c>
     </row>
     <row r="12">
       <c r="F12" s="26" t="s">
         <v>144</v>
       </c>
+      <c r="J12" s="26">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="26" t="s">
         <v>145</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="23"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="J23" s="26">
+        <v>390.08</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="F24" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="J24" s="26">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="F25" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="J25" s="26">
+        <v>12.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="F26" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="J26" s="26" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="I30" s="26" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="s">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A30:H30"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Calcul des valeurs pour r201
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_enzo.xlsx
+++ b/mesures/TP_mesures_enzo.xlsx
@@ -9,6 +9,7 @@
     <sheet state="visible" name="Albrecht" sheetId="4" r:id="rId8"/>
     <sheet state="visible" name="MI" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="TFC" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="r201DOOEngins-ENS" sheetId="7" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -16,12 +17,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="212">
   <si>
     <t>Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
-  </si>
-  <si>
-    <t>Complexité cyclomatique (CC) - iqsort0</t>
   </si>
   <si>
     <t>Score UFC</t>
@@ -30,34 +28,25 @@
     <t>Métriques de Halstead - iqsort0</t>
   </si>
   <si>
-    <t>Périmètre</t>
+    <t>Complexité cyclomatique (CC) - iqsort0</t>
   </si>
   <si>
     <t>Catégorie</t>
   </si>
   <si>
-    <t>Nœuds</t>
-  </si>
-  <si>
-    <t>Fichiers</t>
-  </si>
-  <si>
-    <t>LOC (lignes non vides)</t>
+    <t>Périmètre</t>
   </si>
   <si>
     <t>Opérateurs</t>
   </si>
   <si>
-    <t>LOC moyen / fichier</t>
+    <t>Nœuds</t>
   </si>
   <si>
-    <t>Dépôt complet (script scriptligne.sh)</t>
+    <t>Calcul</t>
   </si>
   <si>
-    <t>Arêtes</t>
-  </si>
-  <si>
-    <t>Calcul de V(G) = E - N + 2P</t>
+    <t>Sous-total</t>
   </si>
   <si>
     <t>Opérandes</t>
@@ -66,7 +55,43 @@
     <t>Mesures</t>
   </si>
   <si>
+    <t>Poids (simple / moyen / difficile)</t>
+  </si>
+  <si>
+    <t>Arêtes</t>
+  </si>
+  <si>
+    <t>Scores (simple / moyen / difficile)</t>
+  </si>
+  <si>
+    <t>Calcul de V(G) = E - N + 2P</t>
+  </si>
+  <si>
+    <t>Opérateur</t>
+  </si>
+  <si>
+    <t>Entrées externes</t>
+  </si>
+  <si>
+    <t>Fichiers</t>
+  </si>
+  <si>
+    <t>Occurrences</t>
+  </si>
+  <si>
+    <t>LOC (lignes non vides)</t>
+  </si>
+  <si>
     <t>Nœud</t>
+  </si>
+  <si>
+    <t>Opérande</t>
+  </si>
+  <si>
+    <t>3×4 + 4×3 + 6×1</t>
+  </si>
+  <si>
+    <t>LOC moyen / fichier</t>
   </si>
   <si>
     <t>Instruction</t>
@@ -75,43 +100,10 @@
     <t>Lignes</t>
   </si>
   <si>
-    <t>Opérateur</t>
-  </si>
-  <si>
-    <t>De</t>
-  </si>
-  <si>
-    <t>Vers</t>
-  </si>
-  <si>
-    <t>Occurrences</t>
-  </si>
-  <si>
-    <t>Opérande</t>
-  </si>
-  <si>
-    <t>E (arêtes)</t>
-  </si>
-  <si>
     <t>nt (opérateurs distincts)</t>
   </si>
   <si>
-    <t>Calcul</t>
-  </si>
-  <si>
-    <t>Sous-total</t>
-  </si>
-  <si>
-    <t>Poids (simple / moyen / difficile)</t>
-  </si>
-  <si>
-    <t>Scores (simple / moyen / difficile)</t>
-  </si>
-  <si>
-    <t>Entrées externes</t>
-  </si>
-  <si>
-    <t>3×4 + 4×3 + 6×1</t>
+    <t>Dépôt complet (script scriptligne.sh)</t>
   </si>
   <si>
     <t>1 / 2 / 4</t>
@@ -120,49 +112,31 @@
     <t>1 / 1 / 0</t>
   </si>
   <si>
-    <t>void</t>
+    <t>De</t>
   </si>
   <si>
     <t>1×1 + 2×1 + 4×0</t>
   </si>
   <si>
-    <t>N1</t>
+    <t>Vers</t>
   </si>
   <si>
     <t>Sorties externes</t>
   </si>
   <si>
-    <t>iqsort0</t>
-  </si>
-  <si>
-    <t>if (n &lt;= 1)</t>
-  </si>
-  <si>
     <t>4×0 + 5×2 + 7×1</t>
   </si>
   <si>
-    <t>3-4</t>
-  </si>
-  <si>
-    <t>Nt (occurrences d'opérateurs)</t>
+    <t>E (arêtes)</t>
   </si>
   <si>
     <t>2 / 3 / 5</t>
   </si>
   <si>
-    <t>N2</t>
-  </si>
-  <si>
     <t>0 / 1 / 0</t>
   </si>
   <si>
-    <t>N (nœuds)</t>
-  </si>
-  <si>
     <t>2×0 + 3×1 + 5×0</t>
-  </si>
-  <si>
-    <t>Application ./app (php, js, jsx, css, ps1)</t>
   </si>
   <si>
     <t>Requêtes externes</t>
@@ -174,13 +148,7 @@
     <t>0 / 0 / 0</t>
   </si>
   <si>
-    <t>Écart (Maquette, lockfile, etc.)</t>
-  </si>
-  <si>
     <t>1×0 + 2×0 + 4×0</t>
-  </si>
-  <si>
-    <t>( )</t>
   </si>
   <si>
     <t>Fichiers internes</t>
@@ -189,28 +157,10 @@
     <t>7×3 + 10×0 + 15×0</t>
   </si>
   <si>
-    <t>swap</t>
-  </si>
-  <si>
-    <t>return</t>
-  </si>
-  <si>
     <t>3 / 5 / 8</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>nd (opérandes distincts)</t>
-  </si>
-  <si>
-    <t>N3</t>
-  </si>
-  <si>
     <t>3×0 + 5×0 + 0×0</t>
-  </si>
-  <si>
-    <t>P (composantes connexes)</t>
   </si>
   <si>
     <t>Fichiers externes</t>
@@ -219,44 +169,112 @@
     <t>5×0 + 7×5 + 10×2</t>
   </si>
   <si>
+    <t xml:space="preserve">
+3 / 5 / 8</t>
+  </si>
+  <si>
+    <t>3×0 + 5×0 + 8×0</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
+Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
+Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
+  </si>
+  <si>
+    <t>void</t>
+  </si>
+  <si>
+    <t>iqsort0</t>
+  </si>
+  <si>
+    <t>Nt (occurrences d'opérateurs)</t>
+  </si>
+  <si>
+    <t>N1</t>
+  </si>
+  <si>
+    <t>if (n &lt;= 1)</t>
+  </si>
+  <si>
+    <t>3-4</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>N (nœuds)</t>
+  </si>
+  <si>
+    <t>Application ./app (php, js, jsx, css, ps1)</t>
+  </si>
+  <si>
+    <t>( )</t>
+  </si>
+  <si>
+    <t>Écart (Maquette, lockfile, etc.)</t>
+  </si>
+  <si>
+    <t>swap</t>
+  </si>
+  <si>
+    <t>nd (opérandes distincts)</t>
+  </si>
+  <si>
+    <t>return</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>N3</t>
+  </si>
+  <si>
+    <t>P (composantes connexes)</t>
+  </si>
+  <si>
     <t>i = 1, j = 0</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
-    <t xml:space="preserve">
-3 / 5 / 8</t>
+    <t>int</t>
   </si>
   <si>
     <t>N9</t>
   </si>
   <si>
-    <t>3×0 + 5×0 + 8×0</t>
-  </si>
-  <si>
     <t>V(G) = E - N + 2P</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>Total</t>
   </si>
   <si>
     <t>a</t>
   </si>
   <si>
-    <t>Nd (occurrences d'opérandes)</t>
+    <t>Méthode et hypothèses</t>
   </si>
   <si>
-    <t>Méthode et hypothèses</t>
+    <t>Nd (occurrences d'opérandes)</t>
   </si>
   <si>
     <t>LOC = lignes non vides (commentaires inclus), mesurées avec le script bash scriptligne.sh.</t>
   </si>
   <si>
     <t>Dépôt complet : exclut seulement .git, node_modules, .venv, __pycache__ (fichiers binaires ignorés).</t>
+  </si>
+  <si>
+    <t>Application : find ./app sur *.php, *.js, *.jsx, *.css, *.ps1, hors node_modules et vendor.</t>
+  </si>
+  <si>
+    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
+  </si>
+  <si>
+    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
+  </si>
+  <si>
+    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
   </si>
   <si>
     <t>*</t>
@@ -268,19 +286,13 @@
     <t>N4</t>
   </si>
   <si>
+    <t>Longueur N = Nt + Nd</t>
+  </si>
+  <si>
     <t>i &lt; n ?</t>
   </si>
   <si>
-    <t>Application : find ./app sur *.php, *.js, *.jsx, *.css, *.ps1, hors node_modules et vendor.</t>
-  </si>
-  <si>
-    <t>Longueur N = Nt + Nd</t>
-  </si>
-  <si>
     <t>Contrôle : décisions + 1 (3 décisions : lignes 4, 6, 7)</t>
-  </si>
-  <si>
-    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
   </si>
   <si>
     <t>N5</t>
@@ -289,18 +301,7 @@
     <t>a[i] &lt; a[0] ?</t>
   </si>
   <si>
-    <t>Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
-Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
-Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
-  </si>
-  <si>
     <t>7</t>
-  </si>
-  <si>
-    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
-  </si>
-  <si>
-    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
   </si>
   <si>
     <t>N6</t>
@@ -318,22 +319,22 @@
     <t>N8</t>
   </si>
   <si>
+    <t>Contrôle : écart avec V(G)</t>
+  </si>
+  <si>
     <t>i</t>
   </si>
   <si>
-    <t>Contrôle : écart avec V(G)</t>
-  </si>
-  <si>
     <t>Vocabulaire n = nt + nd</t>
-  </si>
-  <si>
-    <t>{ }</t>
   </si>
   <si>
     <t>N7</t>
   </si>
   <si>
     <t>i++</t>
+  </si>
+  <si>
+    <t>{ }</t>
   </si>
   <si>
     <t>j</t>
@@ -644,6 +645,42 @@
   <si>
     <t>TFC = 0,65 + 0,01 × somme</t>
   </si>
+  <si>
+    <t>Analyse r201DOOEngins-ENS</t>
+  </si>
+  <si>
+    <t>LOC</t>
+  </si>
+  <si>
+    <t>229 (276 lignes physiques, 47 vides, 47 de commentaires, 182 de code pur)</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>total 40 sur 34 méthodes, moyenne 1,18, maximum 4</t>
+  </si>
+  <si>
+    <t>Halstead</t>
+  </si>
+  <si>
+    <t>nt = 33, Nt = 625, nd = 90, Nd = 271, N = 896, n = 123, Volume ≈ 6 220, Difficulté ≈ 49,7, Effort ≈ 309 055</t>
+  </si>
+  <si>
+    <t>MI moyen</t>
+  </si>
+  <si>
+    <t>UFC</t>
+  </si>
+  <si>
+    <t>4 (lecture stricte) ou 14 (lecture « pédagogique »)</t>
+  </si>
+  <si>
+    <t>TFC</t>
+  </si>
+  <si>
+    <t>0,73 (somme des notes = 8)</t>
+  </si>
 </sst>
 </file>
 
@@ -677,6 +714,10 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -684,10 +725,6 @@
     <font>
       <sz val="11.0"/>
       <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -748,7 +785,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -759,39 +796,33 @@
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -800,13 +831,19 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -817,7 +854,7 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -831,6 +868,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -861,6 +901,10 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1089,54 +1133,54 @@
       <c r="D2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
+      <c r="A3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="6">
+      <c r="A4" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="9">
         <v>301.0</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="10">
         <v>23053.0</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="16">
         <f>C4/B4</f>
         <v>76.58803987</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="8">
+      <c r="A5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="10">
         <v>13696.0</v>
       </c>
-      <c r="D5" s="5"/>
+      <c r="D5" s="8"/>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="12">
+      <c r="A6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="17">
         <f>C4-C5</f>
         <v>9357</v>
       </c>
-      <c r="D6" s="5"/>
+      <c r="D6" s="8"/>
     </row>
     <row r="7">
       <c r="A7" s="2"/>
@@ -1153,48 +1197,48 @@
       <c r="D8" s="2"/>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="5" t="s">
-        <v>78</v>
+      <c r="A9" s="8" t="s">
+        <v>79</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="5" t="s">
-        <v>79</v>
+      <c r="A10" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="5" t="s">
-        <v>84</v>
+      <c r="A11" s="8" t="s">
+        <v>81</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="5" t="s">
-        <v>87</v>
+      <c r="A12" s="8" t="s">
+        <v>82</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>92</v>
+      <c r="A13" s="8" t="s">
+        <v>83</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
     </row>
     <row r="14" ht="15.0" customHeight="1">
-      <c r="A14" s="5" t="s">
-        <v>93</v>
+      <c r="A14" s="8" t="s">
+        <v>84</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -7144,7 +7188,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7168,118 +7212,118 @@
     </row>
     <row r="3" ht="15.0" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I3" s="2"/>
     </row>
     <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
+      <c r="A4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>21</v>
+      <c r="E4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="5">
+      <c r="H4" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="8">
         <f>COUNTA(E5:E15)</f>
         <v>11</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>41</v>
+      <c r="A5" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>59</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>44</v>
+      <c r="E5" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>60</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="I5" s="5">
+      <c r="H5" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="8">
         <f>COUNTA(A5:A13)</f>
         <v>9</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="A6" s="9" t="s">
         <v>60</v>
       </c>
+      <c r="B6" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>68</v>
+      </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>62</v>
+      <c r="E6" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="I6" s="6">
+      <c r="H6" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="I6" s="9">
         <v>1.0</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>68</v>
+      <c r="A7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>72</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>70</v>
+      <c r="E7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I7" s="4">
         <f>I4-I5+2*I6</f>
@@ -7287,92 +7331,92 @@
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>68</v>
+      <c r="A8" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>72</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>82</v>
+      <c r="E8" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>87</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="I8" s="6">
+      <c r="H8" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="I8" s="9">
         <v>4.0</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="A9" s="9" t="s">
         <v>91</v>
       </c>
+      <c r="B9" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>93</v>
+      </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>88</v>
+      <c r="E9" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>91</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="9" t="s">
         <v>96</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F10" s="6" t="s">
+      <c r="E10" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>98</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="I10" s="5">
+      <c r="H10" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="I10" s="8">
         <f>I7-I8</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>68</v>
+      <c r="C11" s="9" t="s">
+        <v>72</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F11" s="6" t="s">
+      <c r="E11" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>94</v>
       </c>
       <c r="G11" s="2"/>
@@ -7380,21 +7424,21 @@
       <c r="I11" s="2"/>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="9" t="s">
         <v>108</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>103</v>
+      <c r="E12" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>102</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="4" t="s">
@@ -7403,24 +7447,24 @@
       <c r="I12" s="2"/>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B13" s="6" t="s">
+      <c r="A13" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="9" t="s">
         <v>111</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>103</v>
+      <c r="F13" s="9" t="s">
+        <v>102</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="8" t="s">
         <v>112</v>
       </c>
       <c r="I13" s="2"/>
@@ -7430,14 +7474,14 @@
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>82</v>
+      <c r="E14" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>87</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="8" t="s">
         <v>113</v>
       </c>
       <c r="I14" s="2"/>
@@ -7447,14 +7491,14 @@
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>70</v>
+      <c r="F15" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G15" s="2"/>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="8" t="s">
         <v>114</v>
       </c>
       <c r="I15" s="2"/>
@@ -7467,7 +7511,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="5" t="s">
+      <c r="H16" s="8" t="s">
         <v>115</v>
       </c>
       <c r="I16" s="2"/>
@@ -18324,7 +18368,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -18346,174 +18390,174 @@
     </row>
     <row r="3" ht="15.0" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H3" s="2"/>
     </row>
     <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="2"/>
+      <c r="D4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>22</v>
+      <c r="E4" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="G4" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" s="5">
+      <c r="G4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="8">
         <f>COUNTA(A5:A21)</f>
         <v>17</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="6">
+      <c r="A5" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="9">
         <v>1.0</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="6">
+      <c r="D5" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="9">
         <v>3.0</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="H5" s="5">
+      <c r="G5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="8">
         <f>SUM(B5:B21)</f>
         <v>48</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="6">
+      <c r="A6" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="9">
         <v>8.0</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E6" s="6">
+      <c r="D6" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="9">
         <v>2.0</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="G6" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" s="5">
+      <c r="G6" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H6" s="8">
         <f>COUNTA(D5:D12)</f>
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="9">
         <v>3.0</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="6">
+      <c r="D7" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="9">
         <v>7.0</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="G7" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H7" s="5">
+      <c r="G7" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H7" s="8">
         <f>SUM(E5:E12)</f>
         <v>36</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="6">
+      <c r="A8" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="9">
         <v>1.0</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" s="6">
+      <c r="D8" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" s="9">
         <v>4.0</v>
       </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="H8" s="5">
+      <c r="G8" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H8" s="8">
         <f>H5+H7</f>
         <v>84</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="9">
         <v>9.0</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E9" s="6">
+      <c r="D9" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="9">
         <v>6.0</v>
       </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="8">
         <f>H4+H6</f>
         <v>25</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B10" s="6">
+      <c r="A10" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="9">
         <v>1.0</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="9">
         <v>7.0</v>
       </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="8" t="s">
         <v>106</v>
       </c>
       <c r="H10" s="18">
@@ -18522,21 +18566,21 @@
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="9">
         <v>8.0</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="9">
         <v>3.0</v>
       </c>
       <c r="F11" s="2"/>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="8" t="s">
         <v>118</v>
       </c>
       <c r="H11" s="18">
@@ -18545,21 +18589,21 @@
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="9">
         <v>2.0</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="9">
         <v>4.0</v>
       </c>
       <c r="F12" s="2"/>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="8" t="s">
         <v>121</v>
       </c>
       <c r="H12" s="19">
@@ -18568,10 +18612,10 @@
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="9">
         <v>1.0</v>
       </c>
       <c r="C13" s="2"/>
@@ -18582,10 +18626,10 @@
       <c r="H13" s="2"/>
     </row>
     <row r="14" ht="15.0" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="6">
+      <c r="A14" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="9">
         <v>1.0</v>
       </c>
       <c r="C14" s="2"/>
@@ -18598,106 +18642,106 @@
       <c r="H14" s="2"/>
     </row>
     <row r="15" ht="15.0" customHeight="1">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="9">
         <v>1.0</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="8" t="s">
         <v>125</v>
       </c>
       <c r="H15" s="2"/>
     </row>
     <row r="16" ht="15.0" customHeight="1">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="9">
         <v>2.0</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="5" t="s">
+      <c r="G16" s="8" t="s">
         <v>127</v>
       </c>
       <c r="H16" s="2"/>
     </row>
     <row r="17" ht="15.0" customHeight="1">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="9">
         <v>2.0</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="5" t="s">
+      <c r="G17" s="8" t="s">
         <v>129</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="6">
+      <c r="B18" s="9">
         <v>2.0</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="5" t="s">
+      <c r="G18" s="8" t="s">
         <v>131</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" ht="15.0" customHeight="1">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="9">
         <v>2.0</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="G19" s="5" t="s">
+      <c r="G19" s="8" t="s">
         <v>133</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="9">
         <v>2.0</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-      <c r="G20" s="5" t="s">
+      <c r="G20" s="8" t="s">
         <v>115</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="9">
         <v>2.0</v>
       </c>
       <c r="C21" s="2"/>
@@ -18723,12 +18767,12 @@
       <c r="H23" s="23"/>
     </row>
     <row r="24" ht="63.75" customHeight="1">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="15" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="25" ht="36.0" customHeight="1">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="15" t="s">
         <v>138</v>
       </c>
     </row>
@@ -28456,234 +28500,234 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="I3" s="9" t="s">
+      <c r="A3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="7">
+        <v>30.0</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="s">
+      <c r="I4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="10">
-        <v>30.0</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="10" t="s">
+      <c r="K4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="L4" s="10" t="s">
+      <c r="M4" s="7">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="M4" s="10">
+      <c r="C5" s="7">
+        <v>17.0</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5" s="7">
         <v>3.0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="10" t="s">
+    <row r="6">
+      <c r="A6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="10">
-        <v>17.0</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="H5" s="10" t="s">
+      <c r="B6" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="7">
+        <v>21.0</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="L6" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="M6" s="7">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="K5" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="L5" s="10" t="s">
+      <c r="C7" s="7">
+        <v>21.0</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="L7" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="M5" s="10">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="s">
+      <c r="M7" s="7">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="C8" s="7">
+        <v>55.0</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="10">
-        <v>21.0</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" s="10" t="s">
+      <c r="I8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="L8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="L6" s="10" t="s">
+      <c r="M8" s="7">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="12"/>
+      <c r="C9" s="13">
+        <v>144.0</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="13"/>
+      <c r="K9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="L9" s="12"/>
+      <c r="M9" s="13">
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="10">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="10">
-        <v>21.0</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="M7" s="10">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C8" s="10">
-        <v>55.0</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="I8" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="L8" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="M8" s="10">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="15">
-        <v>144.0</v>
-      </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15"/>
-      <c r="K9" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="L9" s="14"/>
-      <c r="M9" s="15">
-        <v>6.0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="s">
-        <v>90</v>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
     </row>
     <row r="13">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
     </row>
     <row r="14">
-      <c r="A14" s="16"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
     </row>
     <row r="15">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -28707,7 +28751,7 @@
     </row>
     <row r="7">
       <c r="A7" s="25" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
@@ -28850,19 +28894,19 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="3" t="s">
         <v>156</v>
       </c>
     </row>
@@ -29105,28 +29149,105 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16"/>
+      <c r="A22" s="14"/>
       <c r="B22" s="27" t="s">
         <v>198</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="14">
         <f>SUM(C2:C15)</f>
         <v>23</v>
       </c>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
     </row>
     <row r="23">
-      <c r="A23" s="16"/>
+      <c r="A23" s="14"/>
       <c r="B23" s="27" t="s">
         <v>199</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="14">
         <f>0.65+0.01*C16</f>
         <v>0.67</v>
       </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29">
+        <v>112.24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="s">
+        <v>211</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Ajout q14, couplage et manque de cohésion
</commit_message>
<xml_diff>
--- a/mesures/TP_mesures_enzo.xlsx
+++ b/mesures/TP_mesures_enzo.xlsx
@@ -10,6 +10,7 @@
     <sheet state="visible" name="MI" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="TFC" sheetId="6" r:id="rId10"/>
     <sheet state="visible" name="r201DOOEngins-ENS" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="Couplage-Cohésion" sheetId="8" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -17,81 +18,66 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="233">
   <si>
     <t>Mesure LOC (Lines Of Code) - projet BAGNIS-MARCUS-PIBOULEAU</t>
   </si>
   <si>
-    <t>Score UFC</t>
+    <t>Périmètre</t>
   </si>
   <si>
-    <t>Métriques de Halstead - iqsort0</t>
+    <t>Fichiers</t>
+  </si>
+  <si>
+    <t>LOC (lignes non vides)</t>
+  </si>
+  <si>
+    <t>LOC moyen / fichier</t>
+  </si>
+  <si>
+    <t>Dépôt complet (script scriptligne.sh)</t>
+  </si>
+  <si>
+    <t>Application ./app (php, js, jsx, css, ps1)</t>
+  </si>
+  <si>
+    <t>Écart (Maquette, lockfile, etc.)</t>
+  </si>
+  <si>
+    <t>Méthode et hypothèses</t>
+  </si>
+  <si>
+    <t>LOC = lignes non vides (commentaires inclus), mesurées avec le script bash scriptligne.sh.</t>
+  </si>
+  <si>
+    <t>Dépôt complet : exclut seulement .git, node_modules, .venv, __pycache__ (fichiers binaires ignorés).</t>
+  </si>
+  <si>
+    <t>Application : find ./app sur *.php, *.js, *.jsx, *.css, *.ps1, hors node_modules et vendor.</t>
+  </si>
+  <si>
+    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
+  </si>
+  <si>
+    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
+  </si>
+  <si>
+    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
   </si>
   <si>
     <t>Complexité cyclomatique (CC) - iqsort0</t>
   </si>
   <si>
-    <t>Catégorie</t>
-  </si>
-  <si>
-    <t>Périmètre</t>
-  </si>
-  <si>
-    <t>Opérateurs</t>
-  </si>
-  <si>
     <t>Nœuds</t>
-  </si>
-  <si>
-    <t>Calcul</t>
-  </si>
-  <si>
-    <t>Sous-total</t>
-  </si>
-  <si>
-    <t>Opérandes</t>
-  </si>
-  <si>
-    <t>Mesures</t>
-  </si>
-  <si>
-    <t>Poids (simple / moyen / difficile)</t>
   </si>
   <si>
     <t>Arêtes</t>
   </si>
   <si>
-    <t>Scores (simple / moyen / difficile)</t>
-  </si>
-  <si>
     <t>Calcul de V(G) = E - N + 2P</t>
   </si>
   <si>
-    <t>Opérateur</t>
-  </si>
-  <si>
-    <t>Entrées externes</t>
-  </si>
-  <si>
-    <t>Fichiers</t>
-  </si>
-  <si>
-    <t>Occurrences</t>
-  </si>
-  <si>
-    <t>LOC (lignes non vides)</t>
-  </si>
-  <si>
     <t>Nœud</t>
-  </si>
-  <si>
-    <t>Opérande</t>
-  </si>
-  <si>
-    <t>3×4 + 4×3 + 6×1</t>
-  </si>
-  <si>
-    <t>LOC moyen / fichier</t>
   </si>
   <si>
     <t>Instruction</t>
@@ -100,97 +86,13 @@
     <t>Lignes</t>
   </si>
   <si>
-    <t>nt (opérateurs distincts)</t>
-  </si>
-  <si>
-    <t>Dépôt complet (script scriptligne.sh)</t>
-  </si>
-  <si>
-    <t>1 / 2 / 4</t>
-  </si>
-  <si>
-    <t>1 / 1 / 0</t>
-  </si>
-  <si>
     <t>De</t>
-  </si>
-  <si>
-    <t>1×1 + 2×1 + 4×0</t>
   </si>
   <si>
     <t>Vers</t>
   </si>
   <si>
-    <t>Sorties externes</t>
-  </si>
-  <si>
-    <t>4×0 + 5×2 + 7×1</t>
-  </si>
-  <si>
     <t>E (arêtes)</t>
-  </si>
-  <si>
-    <t>2 / 3 / 5</t>
-  </si>
-  <si>
-    <t>0 / 1 / 0</t>
-  </si>
-  <si>
-    <t>2×0 + 3×1 + 5×0</t>
-  </si>
-  <si>
-    <t>Requêtes externes</t>
-  </si>
-  <si>
-    <t>3×7 + 4×0 + 6×0</t>
-  </si>
-  <si>
-    <t>0 / 0 / 0</t>
-  </si>
-  <si>
-    <t>1×0 + 2×0 + 4×0</t>
-  </si>
-  <si>
-    <t>Fichiers internes</t>
-  </si>
-  <si>
-    <t>7×3 + 10×0 + 15×0</t>
-  </si>
-  <si>
-    <t>3 / 5 / 8</t>
-  </si>
-  <si>
-    <t>3×0 + 5×0 + 0×0</t>
-  </si>
-  <si>
-    <t>Fichiers externes</t>
-  </si>
-  <si>
-    <t>5×0 + 7×5 + 10×2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-3 / 5 / 8</t>
-  </si>
-  <si>
-    <t>3×0 + 5×0 + 8×0</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
-Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
-Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
-  </si>
-  <si>
-    <t>void</t>
-  </si>
-  <si>
-    <t>iqsort0</t>
-  </si>
-  <si>
-    <t>Nt (occurrences d'opérateurs)</t>
   </si>
   <si>
     <t>N1</t>
@@ -206,21 +108,6 @@
   </si>
   <si>
     <t>N (nœuds)</t>
-  </si>
-  <si>
-    <t>Application ./app (php, js, jsx, css, ps1)</t>
-  </si>
-  <si>
-    <t>( )</t>
-  </si>
-  <si>
-    <t>Écart (Maquette, lockfile, etc.)</t>
-  </si>
-  <si>
-    <t>swap</t>
-  </si>
-  <si>
-    <t>nd (opérandes distincts)</t>
   </si>
   <si>
     <t>return</t>
@@ -241,52 +128,13 @@
     <t>6</t>
   </si>
   <si>
-    <t>int</t>
-  </si>
-  <si>
     <t>N9</t>
   </si>
   <si>
     <t>V(G) = E - N + 2P</t>
   </si>
   <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>Méthode et hypothèses</t>
-  </si>
-  <si>
-    <t>Nd (occurrences d'opérandes)</t>
-  </si>
-  <si>
-    <t>LOC = lignes non vides (commentaires inclus), mesurées avec le script bash scriptligne.sh.</t>
-  </si>
-  <si>
-    <t>Dépôt complet : exclut seulement .git, node_modules, .venv, __pycache__ (fichiers binaires ignorés).</t>
-  </si>
-  <si>
-    <t>Application : find ./app sur *.php, *.js, *.jsx, *.css, *.ps1, hors node_modules et vendor.</t>
-  </si>
-  <si>
-    <t>Le dépôt complet inclut pnpm-lock.yaml (1077 lignes, fichier généré) et la Maquette (prototype).</t>
-  </si>
-  <si>
-    <t>Les valeurs en bleu sont des résultats saisis depuis le terminal ; les valeurs en noir sont des formules.</t>
-  </si>
-  <si>
-    <t>Le périmètre ./app exclut .html, .sql, .json, .md, .yml.</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
     <t>N4</t>
-  </si>
-  <si>
-    <t>Longueur N = Nt + Nd</t>
   </si>
   <si>
     <t>i &lt; n ?</t>
@@ -313,34 +161,16 @@
     <t>8</t>
   </si>
   <si>
-    <t>,</t>
-  </si>
-  <si>
     <t>N8</t>
   </si>
   <si>
     <t>Contrôle : écart avec V(G)</t>
   </si>
   <si>
-    <t>i</t>
-  </si>
-  <si>
-    <t>Vocabulaire n = nt + nd</t>
-  </si>
-  <si>
     <t>N7</t>
   </si>
   <si>
     <t>i++</t>
-  </si>
-  <si>
-    <t>{ }</t>
-  </si>
-  <si>
-    <t>j</t>
-  </si>
-  <si>
-    <t>Volume = N * log2(n)</t>
   </si>
   <si>
     <t>swap + 2 appels iqsort0</t>
@@ -368,6 +198,84 @@
   </si>
   <si>
     <t>Valeurs en bleu : saisies ; valeurs en noir : formules.</t>
+  </si>
+  <si>
+    <t>Métriques de Halstead - iqsort0</t>
+  </si>
+  <si>
+    <t>Opérateurs</t>
+  </si>
+  <si>
+    <t>Opérandes</t>
+  </si>
+  <si>
+    <t>Mesures</t>
+  </si>
+  <si>
+    <t>Opérateur</t>
+  </si>
+  <si>
+    <t>Occurrences</t>
+  </si>
+  <si>
+    <t>Opérande</t>
+  </si>
+  <si>
+    <t>nt (opérateurs distincts)</t>
+  </si>
+  <si>
+    <t>void</t>
+  </si>
+  <si>
+    <t>iqsort0</t>
+  </si>
+  <si>
+    <t>Nt (occurrences d'opérateurs)</t>
+  </si>
+  <si>
+    <t>( )</t>
+  </si>
+  <si>
+    <t>swap</t>
+  </si>
+  <si>
+    <t>nd (opérandes distincts)</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>Nd (occurrences d'opérandes)</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>Longueur N = Nt + Nd</t>
+  </si>
+  <si>
+    <t>,</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>Vocabulaire n = nt + nd</t>
+  </si>
+  <si>
+    <t>{ }</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>Volume = N * log2(n)</t>
   </si>
   <si>
     <t>;</t>
@@ -437,6 +345,99 @@
   </si>
   <si>
     <t>Or, les compteurs de base sont ambigus, car deux personnes avec le même code peuvent obtenir un résultat différent. On ne peut donc pas dire si les mesures représentent fidèlement ce qu'elles sont censées représenter.</t>
+  </si>
+  <si>
+    <t>Score UFC</t>
+  </si>
+  <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
+    <t>Calcul</t>
+  </si>
+  <si>
+    <t>Sous-total</t>
+  </si>
+  <si>
+    <t>Poids (simple / moyen / difficile)</t>
+  </si>
+  <si>
+    <t>Scores (simple / moyen / difficile)</t>
+  </si>
+  <si>
+    <t>Entrées externes</t>
+  </si>
+  <si>
+    <t>3×4 + 4×3 + 6×1</t>
+  </si>
+  <si>
+    <t>1 / 2 / 4</t>
+  </si>
+  <si>
+    <t>1 / 1 / 0</t>
+  </si>
+  <si>
+    <t>1×1 + 2×1 + 4×0</t>
+  </si>
+  <si>
+    <t>Sorties externes</t>
+  </si>
+  <si>
+    <t>4×0 + 5×2 + 7×1</t>
+  </si>
+  <si>
+    <t>2 / 3 / 5</t>
+  </si>
+  <si>
+    <t>0 / 1 / 0</t>
+  </si>
+  <si>
+    <t>2×0 + 3×1 + 5×0</t>
+  </si>
+  <si>
+    <t>Requêtes externes</t>
+  </si>
+  <si>
+    <t>3×7 + 4×0 + 6×0</t>
+  </si>
+  <si>
+    <t>0 / 0 / 0</t>
+  </si>
+  <si>
+    <t>1×0 + 2×0 + 4×0</t>
+  </si>
+  <si>
+    <t>Fichiers internes</t>
+  </si>
+  <si>
+    <t>7×3 + 10×0 + 15×0</t>
+  </si>
+  <si>
+    <t>3 / 5 / 8</t>
+  </si>
+  <si>
+    <t>3×0 + 5×0 + 0×0</t>
+  </si>
+  <si>
+    <t>Fichiers externes</t>
+  </si>
+  <si>
+    <t>5×0 + 7×5 + 10×2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+3 / 5 / 8</t>
+  </si>
+  <si>
+    <t>3×0 + 5×0 + 8×0</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Pour établir des poids, on part de l'intuition que tous les éléments d'un système ne demandent pas le même travail. Dans un site marchand, un écran d'alerte « saisie incorrecte » se fait en quelques minutes, alors qu'un formulaire de saisie demande des champs, des contrôles et un enregistrement. On les range donc par niveaux (simple, moyen, difficile) en comparant leur complexité.
+Pour chiffrer ces niveaux, on prend un élément simple comme référence, par exemple 3, et on en déduit les autres. Un moyen vaut un peu plus, un difficile à peu près le double. On peut aussi s'appuyer sur le temps réellement passé sur des projets précédents, ou demander l'avis de plusieurs développeurs expérimentés.
+Les poids restent donc en partie subjectifs : ils dépendent de l'équipe et des technologies, et il faut les réajuster au fil des projets.</t>
   </si>
   <si>
     <t>Index of maintenability ( MI )</t>
@@ -681,6 +682,69 @@
   <si>
     <t>0,73 (somme des notes = 8)</t>
   </si>
+  <si>
+    <t>Classe</t>
+  </si>
+  <si>
+    <t>CBO</t>
+  </si>
+  <si>
+    <t>Classes liées</t>
+  </si>
+  <si>
+    <t>Nb méthodes</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>LCOM</t>
+  </si>
+  <si>
+    <t>Carburant</t>
+  </si>
+  <si>
+    <t>Aucune</t>
+  </si>
+  <si>
+    <t>Electrique</t>
+  </si>
+  <si>
+    <t>Propulsion</t>
+  </si>
+  <si>
+    <t>Engin</t>
+  </si>
+  <si>
+    <t>Eolienne</t>
+  </si>
+  <si>
+    <t>Flottant</t>
+  </si>
+  <si>
+    <t>Engin, Propulsion</t>
+  </si>
+  <si>
+    <t>Main</t>
+  </si>
+  <si>
+    <t>Carburant, Electrique, Engin, Flottant, Propulsion, Roulant, Thermique</t>
+  </si>
+  <si>
+    <t>Marker</t>
+  </si>
+  <si>
+    <t>Roulant</t>
+  </si>
+  <si>
+    <t>Thermique</t>
+  </si>
+  <si>
+    <t>Propulsion, Carburant</t>
+  </si>
 </sst>
 </file>
 
@@ -714,10 +778,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -725,6 +785,17 @@
     <font>
       <sz val="11.0"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font/>
+    <font>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -737,13 +808,6 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="12.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font/>
   </fonts>
   <fills count="3">
     <fill>
@@ -796,80 +860,80 @@
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
     <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -905,6 +969,10 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1133,54 +1201,54 @@
       <c r="D2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="15.0" customHeight="1">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="9">
+      <c r="B4" s="5">
         <v>301.0</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="6">
         <v>23053.0</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="7">
         <f>C4/B4</f>
         <v>76.58803987</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="10">
+      <c r="A5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="6">
         <v>13696.0</v>
       </c>
-      <c r="D5" s="8"/>
+      <c r="D5" s="4"/>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="17">
+      <c r="A6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="8">
         <f>C4-C5</f>
         <v>9357</v>
       </c>
-      <c r="D6" s="8"/>
+      <c r="D6" s="4"/>
     </row>
     <row r="7">
       <c r="A7" s="2"/>
@@ -1189,56 +1257,56 @@
       <c r="D7" s="2"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="4" t="s">
-        <v>77</v>
+      <c r="A8" s="9" t="s">
+        <v>8</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="8" t="s">
-        <v>79</v>
+      <c r="A9" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="8" t="s">
-        <v>80</v>
+      <c r="A10" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="8" t="s">
-        <v>81</v>
+      <c r="A11" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="8" t="s">
-        <v>82</v>
+      <c r="A12" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="8" t="s">
-        <v>83</v>
+      <c r="A13" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
     </row>
     <row r="14" ht="15.0" customHeight="1">
-      <c r="A14" s="8" t="s">
-        <v>84</v>
+      <c r="A14" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -7188,7 +7256,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7211,261 +7279,261 @@
       <c r="I2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>7</v>
+      <c r="A3" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="4" t="s">
-        <v>13</v>
+      <c r="E3" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="4" t="s">
-        <v>15</v>
+      <c r="H3" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="I3" s="2"/>
     </row>
     <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>26</v>
-      </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>33</v>
+      <c r="E4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="8">
+      <c r="H4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="4">
         <f>COUNTA(E5:E15)</f>
         <v>11</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>59</v>
+      <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>60</v>
+      <c r="E5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="I5" s="8">
+      <c r="H5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="4">
         <f>COUNTA(A5:A13)</f>
         <v>9</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>68</v>
+      <c r="A6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>69</v>
+      <c r="E6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="I6" s="9">
+      <c r="H6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="5">
         <v>1.0</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>72</v>
+      <c r="A7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>74</v>
+      <c r="E7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I7" s="4">
+      <c r="H7" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="9">
         <f>I4-I5+2*I6</f>
         <v>4</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>72</v>
+      <c r="A8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>87</v>
+      <c r="E8" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="I8" s="9">
+      <c r="H8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" s="5">
         <v>4.0</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>93</v>
+      <c r="A9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>91</v>
+      <c r="E9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>41</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>96</v>
+      <c r="A10" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>46</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>98</v>
+      <c r="E10" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>47</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="I10" s="8">
+      <c r="H10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="4">
         <f>I7-I8</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>72</v>
+      <c r="A11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>94</v>
+      <c r="E11" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>108</v>
+      <c r="A12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>102</v>
+      <c r="E12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="4" t="s">
-        <v>109</v>
+      <c r="H12" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="I12" s="2"/>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>111</v>
+      <c r="A13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>102</v>
+      <c r="E13" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="8" t="s">
-        <v>112</v>
+      <c r="H13" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -7474,15 +7542,15 @@
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>87</v>
+      <c r="E14" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="8" t="s">
-        <v>113</v>
+      <c r="H14" s="4" t="s">
+        <v>57</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -7491,15 +7559,15 @@
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>74</v>
+      <c r="E15" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="G15" s="2"/>
-      <c r="H15" s="8" t="s">
-        <v>114</v>
+      <c r="H15" s="4" t="s">
+        <v>58</v>
       </c>
       <c r="I15" s="2"/>
     </row>
@@ -7511,8 +7579,8 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="8" t="s">
-        <v>115</v>
+      <c r="H16" s="4" t="s">
+        <v>59</v>
       </c>
       <c r="I16" s="2"/>
     </row>
@@ -18368,7 +18436,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -18389,233 +18457,233 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" ht="15.0" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>6</v>
+      <c r="A3" s="9" t="s">
+        <v>61</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
+      <c r="D3" s="9" t="s">
+        <v>62</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="4" t="s">
-        <v>11</v>
+      <c r="G3" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="H3" s="2"/>
     </row>
     <row r="4" ht="15.0" customHeight="1">
-      <c r="A4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>19</v>
+      <c r="A4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>19</v>
+      <c r="D4" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="G4" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="8">
+      <c r="G4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="H4" s="4">
         <f>COUNTA(A5:A21)</f>
         <v>17</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="A5" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="9">
+      <c r="A5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="5">
         <v>1.0</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E5" s="9">
+      <c r="D5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="5">
         <v>3.0</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="8">
+      <c r="G5" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H5" s="4">
         <f>SUM(B5:B21)</f>
         <v>48</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="9">
+      <c r="A6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="5">
         <v>8.0</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" s="9">
+      <c r="D6" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="5">
         <v>2.0</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="G6" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H6" s="8">
+      <c r="G6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="4">
         <f>COUNTA(D5:D12)</f>
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="9">
+      <c r="A7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="5">
         <v>3.0</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="9">
-        <v>7.0</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="H7" s="8">
+      <c r="H7" s="4">
         <f>SUM(E5:E12)</f>
         <v>36</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="9">
+      <c r="A8" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="5">
         <v>1.0</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8" s="9">
+      <c r="D8" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E8" s="5">
         <v>4.0</v>
       </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="H8" s="8">
+      <c r="G8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H8" s="4">
         <f>H5+H7</f>
         <v>84</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
-      <c r="A9" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B9" s="9">
+      <c r="A9" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="5">
         <v>9.0</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="E9" s="9">
+      <c r="D9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="5">
         <v>6.0</v>
       </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="H9" s="8">
+      <c r="G9" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" s="4">
         <f>H4+H6</f>
         <v>25</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B10" s="9">
+      <c r="A10" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="5">
         <v>1.0</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="E10" s="9">
+      <c r="D10" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E10" s="5">
         <v>7.0</v>
       </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="H10" s="18">
+      <c r="G10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" s="10">
         <f>H8*LOG(H9,2)</f>
         <v>390.0839199</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="B11" s="9">
+      <c r="A11" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="5">
         <v>8.0</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="E11" s="9">
+      <c r="D11" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" s="5">
         <v>3.0</v>
       </c>
       <c r="F11" s="2"/>
-      <c r="G11" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="H11" s="18">
+      <c r="G11" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" s="10">
         <f>(H4/2)*(H7/H6)</f>
         <v>38.25</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B12" s="9">
+      <c r="A12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="5">
         <v>2.0</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="E12" s="9">
+      <c r="D12" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="5">
         <v>4.0</v>
       </c>
       <c r="F12" s="2"/>
-      <c r="G12" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="H12" s="19">
+      <c r="G12" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="H12" s="11">
         <f>H11*H10</f>
         <v>14920.70994</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="B13" s="9">
+      <c r="A13" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="5">
         <v>1.0</v>
       </c>
       <c r="C13" s="2"/>
@@ -18626,122 +18694,122 @@
       <c r="H13" s="2"/>
     </row>
     <row r="14" ht="15.0" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B14" s="9">
+      <c r="A14" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="5">
         <v>1.0</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="4" t="s">
-        <v>123</v>
+      <c r="G14" s="9" t="s">
+        <v>93</v>
       </c>
       <c r="H14" s="2"/>
     </row>
     <row r="15" ht="15.0" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="B15" s="9">
+      <c r="A15" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" s="5">
         <v>1.0</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="8" t="s">
-        <v>125</v>
+      <c r="G15" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="H15" s="2"/>
     </row>
     <row r="16" ht="15.0" customHeight="1">
-      <c r="A16" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="B16" s="9">
+      <c r="A16" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="5">
         <v>2.0</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="8" t="s">
-        <v>127</v>
+      <c r="G16" s="4" t="s">
+        <v>97</v>
       </c>
       <c r="H16" s="2"/>
     </row>
     <row r="17" ht="15.0" customHeight="1">
-      <c r="A17" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="B17" s="9">
+      <c r="A17" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" s="5">
         <v>2.0</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="8" t="s">
-        <v>129</v>
+      <c r="G17" s="4" t="s">
+        <v>99</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="9">
+      <c r="A18" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="5">
         <v>2.0</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="8" t="s">
-        <v>131</v>
+      <c r="G18" s="4" t="s">
+        <v>101</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" ht="15.0" customHeight="1">
-      <c r="A19" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="B19" s="9">
+      <c r="A19" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" s="5">
         <v>2.0</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="G19" s="8" t="s">
-        <v>133</v>
+      <c r="G19" s="4" t="s">
+        <v>103</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="B20" s="9">
+      <c r="A20" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B20" s="5">
         <v>2.0</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-      <c r="G20" s="8" t="s">
-        <v>115</v>
+      <c r="G20" s="4" t="s">
+        <v>59</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="B21" s="9">
+      <c r="A21" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="5">
         <v>2.0</v>
       </c>
       <c r="C21" s="2"/>
@@ -18752,28 +18820,28 @@
       <c r="H21" s="2"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="20" t="s">
-        <v>136</v>
+      <c r="A22" s="12" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="21"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="23"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="15"/>
     </row>
     <row r="24" ht="63.75" customHeight="1">
-      <c r="A24" s="15" t="s">
-        <v>137</v>
+      <c r="A24" s="16" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="25" ht="36.0" customHeight="1">
-      <c r="A25" s="15" t="s">
-        <v>138</v>
+      <c r="A25" s="16" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="26" ht="27.75" customHeight="1"/>
@@ -18783,14 +18851,14 @@
     <row r="30" ht="24.75" customHeight="1"/>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="16.5" customHeight="1">
-      <c r="A32" s="24"/>
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2"/>
@@ -28500,234 +28568,234 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>109</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>9</v>
+      <c r="A3" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="L3" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="7">
+      <c r="A4" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="20">
         <v>30.0</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="M4" s="7">
+      <c r="G4" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="K4" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="L4" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="M4" s="20">
         <v>3.0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="7">
+      <c r="A5" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="20">
         <v>17.0</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="M5" s="7">
+      <c r="G5" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="K5" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="L5" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="M5" s="20">
         <v>3.0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="7">
+      <c r="A6" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="20">
         <v>21.0</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M6" s="7">
+      <c r="G6" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="M6" s="20">
         <v>0.0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="7">
+      <c r="A7" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" s="20">
         <v>21.0</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="M7" s="7">
+      <c r="G7" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="L7" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="M7" s="20">
         <v>0.0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="7">
+      <c r="A8" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" s="20">
         <v>55.0</v>
       </c>
-      <c r="G8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="M8" s="7">
+      <c r="G8" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="I8" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="K8" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="L8" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="M8" s="20">
         <v>0.0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13">
+      <c r="A9" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="23">
         <v>144.0</v>
       </c>
-      <c r="G9" s="11"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="13"/>
-      <c r="K9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="L9" s="12"/>
-      <c r="M9" s="13">
+      <c r="G9" s="21"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="23"/>
+      <c r="K9" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="L9" s="22"/>
+      <c r="M9" s="23">
         <v>6.0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="s">
-        <v>53</v>
+      <c r="A11" s="16" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
     </row>
     <row r="13">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
     </row>
     <row r="14">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
     </row>
     <row r="15">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -28751,15 +28819,15 @@
     </row>
     <row r="7">
       <c r="A7" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="23"/>
+        <v>111</v>
+      </c>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="15"/>
     </row>
     <row r="9">
       <c r="A9" s="26" t="s">
@@ -28805,13 +28873,13 @@
       <c r="A20" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="23"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="15"/>
     </row>
     <row r="23">
       <c r="A23" s="26" t="s">
@@ -28863,14 +28931,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A30:H30"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -28894,19 +28962,19 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="18" t="s">
         <v>156</v>
       </c>
     </row>
@@ -29149,28 +29217,28 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14"/>
+      <c r="A22" s="24"/>
       <c r="B22" s="27" t="s">
         <v>198</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="24">
         <f>SUM(C2:C15)</f>
         <v>23</v>
       </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
     </row>
     <row r="23">
-      <c r="A23" s="14"/>
+      <c r="A23" s="24"/>
       <c r="B23" s="27" t="s">
         <v>199</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="24">
         <f>0.65+0.01*C16</f>
         <v>0.67</v>
       </c>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -29190,7 +29258,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="18" t="s">
         <v>201</v>
       </c>
     </row>
@@ -29200,7 +29268,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="18" t="s">
         <v>203</v>
       </c>
     </row>
@@ -29210,7 +29278,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="18" t="s">
         <v>205</v>
       </c>
     </row>
@@ -29220,7 +29288,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="18" t="s">
         <v>207</v>
       </c>
     </row>
@@ -29230,7 +29298,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="18" t="s">
         <v>208</v>
       </c>
     </row>
@@ -29240,13 +29308,278 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="18" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="26" t="s">
         <v>211</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="s">
+        <v>219</v>
+      </c>
+      <c r="B2" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="D2" s="26">
+        <v>3.0</v>
+      </c>
+      <c r="E2" s="26">
+        <v>3.0</v>
+      </c>
+      <c r="F2" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="G2" s="26">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="26" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="D3" s="26">
+        <v>8.0</v>
+      </c>
+      <c r="E3" s="26">
+        <v>22.0</v>
+      </c>
+      <c r="F3" s="26">
+        <v>6.0</v>
+      </c>
+      <c r="G3" s="26">
+        <v>16.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="B4" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" s="26">
+        <v>6.0</v>
+      </c>
+      <c r="E4" s="26">
+        <v>13.0</v>
+      </c>
+      <c r="F4" s="26">
+        <v>2.0</v>
+      </c>
+      <c r="G4" s="26">
+        <v>11.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="B5" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="D5" s="26">
+        <v>2.0</v>
+      </c>
+      <c r="E5" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="F5" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="G5" s="26">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="B6" s="26">
+        <v>2.0</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="D6" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="E6" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="G6" s="26">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="B7" s="26">
+        <v>7.0</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="E7" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="G7" s="26">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="B8" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="D8" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="G8" s="26">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="B9" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="D9" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="E9" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="G9" s="26">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="s">
+        <v>230</v>
+      </c>
+      <c r="B10" s="26">
+        <v>2.0</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="D10" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="E10" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="F10" s="26">
+        <v>0.0</v>
+      </c>
+      <c r="G10" s="26">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="s">
+        <v>231</v>
+      </c>
+      <c r="B11" s="26">
+        <v>2.0</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>232</v>
+      </c>
+      <c r="D11" s="26">
+        <v>8.0</v>
+      </c>
+      <c r="E11" s="26">
+        <v>17.0</v>
+      </c>
+      <c r="F11" s="26">
+        <v>11.0</v>
+      </c>
+      <c r="G11" s="26">
+        <v>6.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>